<commit_message>
started a preliminary layout
</commit_message>
<xml_diff>
--- a/hardware/RO-Instrument BOM.xlsx
+++ b/hardware/RO-Instrument BOM.xlsx
@@ -2135,7 +2135,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G116"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.63"/>
@@ -4587,10 +4587,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.51"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.04"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4899,10 +4899,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q29"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="24.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="26.74"/>
@@ -6266,7 +6266,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="12.66015625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.62"/>

</xml_diff>

<commit_message>
added USB components, updated BOM, marked components that still needs references
</commit_message>
<xml_diff>
--- a/hardware/RO-Instrument BOM.xlsx
+++ b/hardware/RO-Instrument BOM.xlsx
@@ -2135,7 +2135,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G116"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.63"/>
@@ -4118,7 +4118,7 @@
       <c r="C95" s="2" t="s">
         <v>270</v>
       </c>
-      <c r="D95" s="6" t="s">
+      <c r="D95" s="3" t="s">
         <v>306</v>
       </c>
       <c r="E95" s="2" t="s">
@@ -4139,7 +4139,7 @@
       <c r="C96" s="2" t="s">
         <v>309</v>
       </c>
-      <c r="D96" s="6" t="s">
+      <c r="D96" s="3" t="s">
         <v>310</v>
       </c>
       <c r="E96" s="2" t="s">
@@ -4361,7 +4361,7 @@
       <c r="C107" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D107" s="6" t="s">
+      <c r="D107" s="3" t="s">
         <v>348</v>
       </c>
       <c r="E107" s="2" t="s">
@@ -4587,10 +4587,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.04"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.06"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4899,7 +4899,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q29"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.7"/>
@@ -6266,7 +6266,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="12.6796875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.62"/>

</xml_diff>

<commit_message>
assigned usb resistors and capacitors footprints, created a preliminary 3D PCB model
</commit_message>
<xml_diff>
--- a/hardware/RO-Instrument BOM.xlsx
+++ b/hardware/RO-Instrument BOM.xlsx
@@ -2135,7 +2135,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G116"/>
-  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="15.63"/>
@@ -4587,7 +4587,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D25"/>
-  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34.06"/>
@@ -4899,7 +4899,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:Q29"/>
-  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30.7"/>
@@ -6266,7 +6266,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L4"/>
-  <sheetFormatPr defaultColWidth="12.71484375" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.73046875" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14.62"/>

</xml_diff>